<commit_message>
SCRUM-37: Testplan + RTM + TCs
</commit_message>
<xml_diff>
--- a/Docs/Test-Case/RTM.xlsx
+++ b/Docs/Test-Case/RTM.xlsx
@@ -1526,9 +1526,9 @@
           <t>Trung bình</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Có</t>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Không (API-only)</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1536,9 +1536,9 @@
           <t>TC-AUTH-07, TC-AUTH-08, TC-AUTH-09, TC-AUTH-27</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>TC_FE_MGR_11, TC_FE_MGR_12</t>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>TC-AUTH-07,08,09,27, TC_FE_NEG_02 (xác nhận không có UI)</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>

</xml_diff>